<commit_message>
Save changes for Risk Managemnt April
</commit_message>
<xml_diff>
--- a/backend/data/KPI/projects.xlsx
+++ b/backend/data/KPI/projects.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1532,6 +1532,152 @@
         </is>
       </c>
       <c r="Q15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Req Test PP2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>E-Commerce</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Recommendation Engine</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Node.js</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>React</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Payment Gateway</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10</v>
+      </c>
+      <c r="M16" t="n">
+        <v>15000</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>fdfd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>E-Commerce</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Classification Model</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Django</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>React</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Payment Gateway</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>5</v>
+      </c>
+      <c r="M17" t="n">
+        <v>4455</v>
+      </c>
+      <c r="N17" t="n">
+        <v>2</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Well defined</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
         <is>
           <t>High</t>
         </is>

</xml_diff>

<commit_message>
Fix team allocation, auth guard, and remove hardcoded API key
</commit_message>
<xml_diff>
--- a/backend/data/KPI/projects.xlsx
+++ b/backend/data/KPI/projects.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1534,6 +1534,79 @@
       <c r="Q15" t="inlineStr">
         <is>
           <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>pp2</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prediction Model</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Node.js</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>React</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>User Management</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>MERN</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>15</v>
+      </c>
+      <c r="M16" t="n">
+        <v>300000</v>
+      </c>
+      <c r="N16" t="n">
+        <v>2</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Wide</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>

</xml_diff>